<commit_message>
Updated tests to match new output format and new possible metadata input
</commit_message>
<xml_diff>
--- a/tests/data/19135815/final_mutations_report.xlsx
+++ b/tests/data/19135815/final_mutations_report.xlsx
@@ -3472,12 +3472,12 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>319K</t>
+          <t>N319K</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Substitution</t>
+          <t>Marker</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -4856,12 +4856,12 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>400P</t>
+          <t>S400P</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>Substitution</t>
+          <t>Marker</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -7556,12 +7556,12 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>715N</t>
+          <t>S715N</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>Substitution</t>
+          <t>Marker</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -8316,12 +8316,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>400P</t>
+          <t>S400P</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Substitution</t>
+          <t>Marker</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -11640,12 +11640,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>715N</t>
+          <t>S715N</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Substitution</t>
+          <t>Marker</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -15204,12 +15204,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>319K</t>
+          <t>N319K</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Substitution</t>
+          <t>Marker</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">

</xml_diff>